<commit_message>
feat(web): mejoras vista Connect Latam y nueva vista Mantención
- Actualiza connect_talleres.html con mejoras en la vista Connect Latam
- Agrega nueva vista de Mantención en web_app.py
- Actualiza talleres.xlsx con nuevos datos
- Ajustes en app.py y schema.sql asociados

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/talleres.xlsx
+++ b/Data/talleres.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupokaufmann-my.sharepoint.com/personal/samuel_sanchez_grupokaufmann_com/Documents/Documentos/Dev/geoworkshop/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{84FEF986-3621-40BD-A8EA-225A9AAF25E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAB42109-BFF2-4669-B7D3-BC62036A2542}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="8_{84FEF986-3621-40BD-A8EA-225A9AAF25E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{386666D7-1CD9-41BA-9A8F-63C1CAEB8DAF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2581F85A-D1B6-4F42-AD35-348AD0B72821}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="190">
   <si>
     <t>-53.121693,-70.878428</t>
   </si>
@@ -582,6 +582,30 @@
   </si>
   <si>
     <t>=B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZONA </t>
+  </si>
+  <si>
+    <t>NORTE GRANDE</t>
+  </si>
+  <si>
+    <t>NORTE CHICO</t>
+  </si>
+  <si>
+    <t>METROPOLITANA</t>
+  </si>
+  <si>
+    <t>CENTRO</t>
+  </si>
+  <si>
+    <t>SUR</t>
+  </si>
+  <si>
+    <t>EXTREMO SUR</t>
+  </si>
+  <si>
+    <t>METROPOLITANA ORIENTE</t>
   </si>
 </sst>
 </file>
@@ -603,12 +627,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -638,11 +668,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -977,19 +1008,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1ED25C-D677-4908-964F-893928947FC5}">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="88.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.81640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" style="2"/>
+    <col min="4" max="4" width="88.7265625" customWidth="1"/>
+    <col min="5" max="5" width="27.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.90625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>104</v>
       </c>
@@ -1000,19 +1032,22 @@
         <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>105</v>
       </c>
@@ -1023,19 +1058,22 @@
         <v>98</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>106</v>
       </c>
@@ -1046,19 +1084,22 @@
         <v>94</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>107</v>
       </c>
@@ -1069,19 +1110,22 @@
         <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>108</v>
       </c>
@@ -1092,19 +1136,22 @@
         <v>86</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>109</v>
       </c>
@@ -1115,42 +1162,48 @@
         <v>82</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>79</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>78</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>111</v>
       </c>
@@ -1161,19 +1214,22 @@
         <v>74</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>112</v>
       </c>
@@ -1184,19 +1240,22 @@
         <v>70</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>113</v>
       </c>
@@ -1207,19 +1266,22 @@
         <v>66</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>114</v>
       </c>
@@ -1230,20 +1292,23 @@
         <v>62</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>115</v>
       </c>
@@ -1254,19 +1319,22 @@
         <v>58</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>116</v>
       </c>
@@ -1277,42 +1345,48 @@
         <v>54</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" s="3" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="4" t="s">
         <v>51</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>118</v>
       </c>
@@ -1323,19 +1397,22 @@
         <v>46</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" s="3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>119</v>
       </c>
@@ -1346,19 +1423,22 @@
         <v>42</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>120</v>
       </c>
@@ -1369,19 +1449,22 @@
         <v>38</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>121</v>
       </c>
@@ -1392,19 +1475,22 @@
         <v>34</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>122</v>
       </c>
@@ -1415,19 +1501,22 @@
         <v>30</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="H19" s="3" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>123</v>
       </c>
@@ -1438,19 +1527,22 @@
         <v>26</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="H20" s="3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>124</v>
       </c>
@@ -1461,19 +1553,22 @@
         <v>22</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="H21" s="3" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>125</v>
       </c>
@@ -1484,19 +1579,22 @@
         <v>18</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="H22" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>126</v>
       </c>
@@ -1507,19 +1605,22 @@
         <v>14</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>127</v>
       </c>
@@ -1530,19 +1631,22 @@
         <v>10</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="H24" s="3" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>128</v>
       </c>
@@ -1553,19 +1657,22 @@
         <v>6</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="H25" s="3" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>129</v>
       </c>
@@ -1576,15 +1683,18 @@
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="H26" s="3" t="s">
         <v>179</v>
       </c>
     </row>

</xml_diff>